<commit_message>
Update pvdcom results for these runs
</commit_message>
<xml_diff>
--- a/Studies/Journal - Simon Solar captest/plots/2026-08-EPRI_scenarios_SAMresults.xlsx
+++ b/Studies/Journal - Simon Solar captest/plots/2026-08-EPRI_scenarios_SAMresults.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bmirletz\source\repos\pv_repowering\Studies\Journal - Simon Solar captest\plots\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC5D0517-967D-4494-9AAB-F7152701CF12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A93E59ED-9593-4DCF-A4C4-3CC3F4AFB89E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{04F1D575-AB74-4BA9-9193-B5993F01A15B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{04F1D575-AB74-4BA9-9193-B5993F01A15B}"/>
   </bookViews>
   <sheets>
     <sheet name="Simon" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="14">
   <si>
     <t>Year</t>
   </si>
@@ -69,6 +69,15 @@
   </si>
   <si>
     <t>Repair</t>
+  </si>
+  <si>
+    <t>Time stamp</t>
+  </si>
+  <si>
+    <t>Total after-tax returns | ($)</t>
+  </si>
+  <si>
+    <t>After-tax cumulative NPV | ($)</t>
   </si>
 </sst>
 </file>
@@ -398,10 +407,10 @@
                   <c:v>-1.0464800000000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-4.3150899999999996</c:v>
+                  <c:v>-4.3292599999999997</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-1.0450600000000001</c:v>
+                  <c:v>-1.0515300000000001</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>0</c:v>
@@ -509,10 +518,10 @@
                   <c:v>-1.0464800000000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-28.510200000000001</c:v>
+                  <c:v>-23.018799999999999</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-12.5844</c:v>
+                  <c:v>-10.077299999999999</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>2.7426200000000001</c:v>
@@ -620,16 +629,16 @@
                   <c:v>-1.0464800000000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-1.2334099999999999</c:v>
+                  <c:v>-3.6678099999999998</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-0.13131699999999999</c:v>
+                  <c:v>-1.24272</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>1.86574</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1.7992699999999999</c:v>
+                  <c:v>1.7992600000000001</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>1.7311799999999999</c:v>
@@ -1130,10 +1139,10 @@
                   <c:v>-2.1688999999999998</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-3.8310399999999998</c:v>
+                  <c:v>-3.8365</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-4.2001499999999998</c:v>
+                  <c:v>-4.2079000000000004</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1211,49 +1220,49 @@
                   <c:v>-2.1688999999999998</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-13.1509</c:v>
+                  <c:v>-11.035600000000001</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-17.595600000000001</c:v>
+                  <c:v>-14.594799999999999</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-16.7074</c:v>
+                  <c:v>-13.7066</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-15.8955</c:v>
+                  <c:v>-12.8947</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-15.153499999999999</c:v>
+                  <c:v>-12.152699999999999</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-14.4781</c:v>
+                  <c:v>-11.477399999999999</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-13.8637</c:v>
+                  <c:v>-10.8629</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-13.3025</c:v>
+                  <c:v>-10.3018</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-12.7903</c:v>
+                  <c:v>-9.7895000000000003</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-12.322699999999999</c:v>
+                  <c:v>-9.3219600000000007</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>-11.8971</c:v>
+                  <c:v>-8.8963699999999992</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>-11.5099</c:v>
+                  <c:v>-8.5090800000000009</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>-11.156700000000001</c:v>
+                  <c:v>-8.1559500000000007</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>-10.8348</c:v>
+                  <c:v>-7.8340500000000004</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>-10.463699999999999</c:v>
+                  <c:v>-7.4629599999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1331,49 +1340,49 @@
                   <c:v>-2.1688999999999998</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-2.6440000000000001</c:v>
+                  <c:v>-3.5817100000000002</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-2.6903800000000002</c:v>
+                  <c:v>-4.0206400000000002</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-2.0861499999999999</c:v>
+                  <c:v>-3.4164099999999999</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-1.55186</c:v>
+                  <c:v>-2.88212</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-1.08049</c:v>
+                  <c:v>-2.4107500000000002</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-0.66833299999999995</c:v>
+                  <c:v>-1.9985900000000001</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-0.30918499999999999</c:v>
+                  <c:v>-1.63944</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>4.7341499999999995E-3</c:v>
+                  <c:v>-1.32552</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.278115</c:v>
+                  <c:v>-1.0521400000000001</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.51520200000000005</c:v>
+                  <c:v>-0.81505700000000003</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.71884300000000001</c:v>
+                  <c:v>-0.61141599999999996</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.89267600000000003</c:v>
+                  <c:v>-0.437583</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1.0408200000000001</c:v>
+                  <c:v>-0.289439</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1.1660999999999999</c:v>
+                  <c:v>-0.164159</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1.3488199999999999</c:v>
+                  <c:v>1.8563700000000002E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3076,20 +3085,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A66F2B7E-C15E-4BE7-BAE2-4B1EBEE71C1F}">
-  <dimension ref="A1:Z28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Z69"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.77734375" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.7109375" customWidth="1"/>
     <col min="7" max="8" width="13" customWidth="1"/>
-    <col min="12" max="12" width="4.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="4.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9" customWidth="1"/>
-    <col min="17" max="17" width="3.21875" customWidth="1"/>
-    <col min="22" max="22" width="2.77734375" customWidth="1"/>
+    <col min="17" max="17" width="3.28515625" customWidth="1"/>
+    <col min="22" max="22" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>1</v>
       </c>
@@ -3106,7 +3115,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3174,7 +3183,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>0</v>
       </c>
@@ -3255,7 +3264,7 @@
         <v>-13.5573</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -3304,11 +3313,11 @@
       </c>
       <c r="Q4" s="2"/>
       <c r="R4" s="2">
-        <f t="shared" ref="R4:S28" si="3">G4/1000000</f>
+        <f t="shared" ref="R4:R28" si="3">G4/1000000</f>
         <v>-4.4231999999999996</v>
       </c>
       <c r="S4" s="2">
-        <f t="shared" si="3"/>
+        <f>H4/1000000</f>
         <v>-4.4231999999999996</v>
       </c>
       <c r="T4" s="2">
@@ -3336,7 +3345,7 @@
         <v>-3.5956299999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
@@ -3389,7 +3398,7 @@
         <v>-2.5281600000000002</v>
       </c>
       <c r="S5" s="2">
-        <f t="shared" si="3"/>
+        <f>H5/1000000</f>
         <v>-2.5281600000000002</v>
       </c>
       <c r="T5" s="2">
@@ -3409,15 +3418,15 @@
         <v>-1.34165</v>
       </c>
       <c r="Y5" s="3">
-        <f>Y4+O5</f>
+        <f t="shared" ref="Y5:Y14" si="7">Y4+O5</f>
         <v>-1.34165</v>
       </c>
       <c r="Z5" s="3">
-        <f>Z4+P5</f>
+        <f t="shared" ref="Z5:Z14" si="8">Z4+P5</f>
         <v>-1.34165</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>3</v>
       </c>
@@ -3470,7 +3479,7 @@
         <v>-1.5206299999999999</v>
       </c>
       <c r="S6" s="2">
-        <f t="shared" si="3"/>
+        <f>H6/1000000</f>
         <v>-1.5206299999999999</v>
       </c>
       <c r="T6" s="2">
@@ -3490,28 +3499,28 @@
         <v>-3.4720000000000084E-2</v>
       </c>
       <c r="Y6" s="3">
-        <f>Y5+O6</f>
+        <f t="shared" si="7"/>
         <v>-3.4720000000000084E-2</v>
       </c>
       <c r="Z6" s="3">
-        <f>Z5+P6</f>
+        <f t="shared" si="8"/>
         <v>-3.4720000000000084E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>4</v>
       </c>
       <c r="B7" s="1">
         <v>676313</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7">
         <v>676313</v>
       </c>
       <c r="D7" s="1">
         <v>676313</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="1">
         <v>676313</v>
       </c>
       <c r="G7" s="1">
@@ -3551,7 +3560,7 @@
         <v>-1.04257</v>
       </c>
       <c r="S7" s="2">
-        <f t="shared" si="3"/>
+        <f>H7/1000000</f>
         <v>-1.04257</v>
       </c>
       <c r="T7" s="2">
@@ -3571,34 +3580,34 @@
         <v>0.64159299999999997</v>
       </c>
       <c r="Y7" s="3">
-        <f>Y6+O7</f>
+        <f t="shared" si="7"/>
         <v>0.64159299999999997</v>
       </c>
       <c r="Z7" s="3">
-        <f>Z6+P7</f>
+        <f t="shared" si="8"/>
         <v>0.64159299999999997</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
       <c r="B8" s="1">
         <v>522382</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8">
         <v>522382</v>
       </c>
       <c r="D8" s="1">
         <v>522382</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="1">
         <v>522382</v>
       </c>
       <c r="G8" s="1">
         <v>-703987</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8">
         <v>-703987</v>
       </c>
       <c r="I8" s="1">
@@ -3632,7 +3641,7 @@
         <v>-0.70398700000000003</v>
       </c>
       <c r="S8" s="2">
-        <f t="shared" si="3"/>
+        <f>H8/1000000</f>
         <v>-0.70398700000000003</v>
       </c>
       <c r="T8" s="2">
@@ -3652,22 +3661,22 @@
         <v>1.163975</v>
       </c>
       <c r="Y8" s="3">
-        <f>Y7+O8</f>
+        <f t="shared" si="7"/>
         <v>1.163975</v>
       </c>
       <c r="Z8" s="3">
-        <f>Z7+P8</f>
+        <f t="shared" si="8"/>
         <v>1.163975</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>6</v>
       </c>
       <c r="B9" s="1">
         <v>2407.9699999999998</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9">
         <v>2407.9699999999998</v>
       </c>
       <c r="D9" s="1">
@@ -3679,7 +3688,7 @@
       <c r="G9" s="1">
         <v>-702556</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9">
         <v>-702556</v>
       </c>
       <c r="I9" s="1">
@@ -3713,7 +3722,7 @@
         <v>-0.70255599999999996</v>
       </c>
       <c r="S9" s="2">
-        <f t="shared" si="3"/>
+        <f>H9/1000000</f>
         <v>-0.70255599999999996</v>
       </c>
       <c r="T9" s="2">
@@ -3733,22 +3742,22 @@
         <v>1.1663829699999999</v>
       </c>
       <c r="Y9" s="3">
-        <f>Y8+O9</f>
+        <f t="shared" si="7"/>
         <v>1.1663829699999999</v>
       </c>
       <c r="Z9" s="3">
-        <f>Z8+P9</f>
+        <f t="shared" si="8"/>
         <v>1.1663829699999999</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>7</v>
       </c>
       <c r="B10">
         <v>-522389</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="1">
         <v>-522389</v>
       </c>
       <c r="D10">
@@ -3760,13 +3769,13 @@
       <c r="G10" s="1">
         <v>-987222</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10">
         <v>-987222</v>
       </c>
       <c r="I10" s="1">
         <v>-987222</v>
       </c>
-      <c r="J10" s="1">
+      <c r="J10">
         <v>-987222</v>
       </c>
       <c r="L10">
@@ -3794,7 +3803,7 @@
         <v>-0.98722200000000004</v>
       </c>
       <c r="S10" s="2">
-        <f t="shared" si="3"/>
+        <f>H10/1000000</f>
         <v>-0.98722200000000004</v>
       </c>
       <c r="T10" s="2">
@@ -3814,25 +3823,25 @@
         <v>0.64399396999999992</v>
       </c>
       <c r="Y10" s="3">
-        <f>Y9+O10</f>
+        <f t="shared" si="7"/>
         <v>0.64399396999999992</v>
       </c>
       <c r="Z10" s="3">
-        <f>Z9+P10</f>
+        <f t="shared" si="8"/>
         <v>0.64399396999999992</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>8</v>
       </c>
       <c r="B11">
         <v>-691240</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="1">
         <v>-691240</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11">
         <v>-691240</v>
       </c>
       <c r="E11" s="1">
@@ -3875,7 +3884,7 @@
         <v>-1.3326100000000001</v>
       </c>
       <c r="S11" s="2">
-        <f t="shared" si="3"/>
+        <f>H11/1000000</f>
         <v>-1.3326100000000001</v>
       </c>
       <c r="T11" s="2">
@@ -3895,15 +3904,15 @@
         <v>-4.724603000000005E-2</v>
       </c>
       <c r="Y11" s="3">
-        <f>Y10+O11</f>
+        <f t="shared" si="7"/>
         <v>-4.724603000000005E-2</v>
       </c>
       <c r="Z11" s="3">
-        <f>Z10+P11</f>
+        <f t="shared" si="8"/>
         <v>-4.724603000000005E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9</v>
       </c>
@@ -3913,7 +3922,7 @@
       <c r="C12" s="1">
         <v>-865807</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12">
         <v>-865807</v>
       </c>
       <c r="E12" s="1">
@@ -3956,7 +3965,7 @@
         <v>-1.7292799999999999</v>
       </c>
       <c r="S12" s="2">
-        <f t="shared" si="3"/>
+        <f>H12/1000000</f>
         <v>-1.7292799999999999</v>
       </c>
       <c r="T12" s="2">
@@ -3976,15 +3985,15 @@
         <v>-0.91305303000000004</v>
       </c>
       <c r="Y12" s="3">
-        <f>Y11+O12</f>
+        <f t="shared" si="7"/>
         <v>-0.91305303000000004</v>
       </c>
       <c r="Z12" s="3">
-        <f>Z11+P12</f>
+        <f t="shared" si="8"/>
         <v>-0.91305303000000004</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>10</v>
       </c>
@@ -4037,7 +4046,7 @@
         <v>-2.1688999999999998</v>
       </c>
       <c r="S13" s="2">
-        <f t="shared" si="3"/>
+        <f>H13/1000000</f>
         <v>-2.1688999999999998</v>
       </c>
       <c r="T13" s="2">
@@ -4057,15 +4066,15 @@
         <v>-1.9595330300000002</v>
       </c>
       <c r="Y13" s="3">
-        <f>Y12+O13</f>
+        <f t="shared" si="7"/>
         <v>-1.9595330300000002</v>
       </c>
       <c r="Z13" s="3">
-        <f>Z12+P13</f>
+        <f t="shared" si="8"/>
         <v>-1.9595330300000002</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>11</v>
       </c>
@@ -4073,25 +4082,25 @@
         <v>-1233410</v>
       </c>
       <c r="C14" s="1">
-        <v>-1233410</v>
+        <v>-3667810</v>
       </c>
       <c r="D14" s="1">
-        <v>-4315090</v>
+        <v>-4329260</v>
       </c>
       <c r="E14" s="1">
-        <v>-28510200</v>
+        <v>-23018800</v>
       </c>
       <c r="G14" s="1">
         <v>-2644000</v>
       </c>
       <c r="H14" s="1">
-        <v>-2644000</v>
+        <v>-3581710</v>
       </c>
       <c r="I14" s="1">
-        <v>-3831040</v>
+        <v>-3836500</v>
       </c>
       <c r="J14" s="1">
-        <v>-13150900</v>
+        <v>-11035600</v>
       </c>
       <c r="L14">
         <v>11</v>
@@ -4102,15 +4111,15 @@
       </c>
       <c r="N14" s="2">
         <f t="shared" si="0"/>
-        <v>-1.2334099999999999</v>
+        <v>-3.6678099999999998</v>
       </c>
       <c r="O14" s="2">
         <f t="shared" si="1"/>
-        <v>-4.3150899999999996</v>
+        <v>-4.3292599999999997</v>
       </c>
       <c r="P14" s="2">
         <f t="shared" si="2"/>
-        <v>-28.510200000000001</v>
+        <v>-23.018799999999999</v>
       </c>
       <c r="Q14" s="2"/>
       <c r="R14" s="2">
@@ -4118,16 +4127,16 @@
         <v>-2.6440000000000001</v>
       </c>
       <c r="S14" s="2">
-        <f t="shared" si="3"/>
-        <v>-2.6440000000000001</v>
+        <f>H14/1000000</f>
+        <v>-3.5817100000000002</v>
       </c>
       <c r="T14" s="2">
         <f t="shared" si="4"/>
-        <v>-3.8310399999999998</v>
+        <v>-3.8365</v>
       </c>
       <c r="U14" s="2">
         <f t="shared" si="5"/>
-        <v>-13.1509</v>
+        <v>-11.035600000000001</v>
       </c>
       <c r="W14" s="3">
         <f t="shared" si="6"/>
@@ -4135,18 +4144,18 @@
       </c>
       <c r="X14" s="3">
         <f t="shared" si="6"/>
-        <v>-3.1929430300000003</v>
+        <v>-5.6273430300000005</v>
       </c>
       <c r="Y14" s="3">
-        <f>Y13+O14</f>
-        <v>-6.2746230299999999</v>
+        <f t="shared" si="7"/>
+        <v>-6.2887930299999999</v>
       </c>
       <c r="Z14" s="3">
-        <f>Z13+P14</f>
-        <v>-30.46973303</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" si="8"/>
+        <v>-24.978333029999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>12</v>
       </c>
@@ -4154,25 +4163,25 @@
         <v>-131317</v>
       </c>
       <c r="C15" s="1">
-        <v>-131317</v>
+        <v>-1242720</v>
       </c>
       <c r="D15" s="1">
-        <v>-1045060</v>
+        <v>-1051530</v>
       </c>
       <c r="E15" s="1">
-        <v>-12584400</v>
+        <v>-10077300</v>
       </c>
       <c r="G15" s="1">
         <v>-2690380</v>
       </c>
       <c r="H15" s="1">
-        <v>-2690380</v>
+        <v>-4020640</v>
       </c>
       <c r="I15" s="1">
-        <v>-4200150</v>
+        <v>-4207900</v>
       </c>
       <c r="J15" s="1">
-        <v>-17595600</v>
+        <v>-14594800</v>
       </c>
       <c r="L15">
         <v>12</v>
@@ -4183,15 +4192,15 @@
       </c>
       <c r="N15" s="2">
         <f t="shared" si="0"/>
-        <v>-0.13131699999999999</v>
+        <v>-1.24272</v>
       </c>
       <c r="O15" s="2">
         <f t="shared" si="1"/>
-        <v>-1.0450600000000001</v>
+        <v>-1.0515300000000001</v>
       </c>
       <c r="P15" s="2">
         <f t="shared" si="2"/>
-        <v>-12.5844</v>
+        <v>-10.077299999999999</v>
       </c>
       <c r="Q15" s="2"/>
       <c r="R15" s="2">
@@ -4199,35 +4208,35 @@
         <v>-2.6903800000000002</v>
       </c>
       <c r="S15" s="2">
-        <f t="shared" si="3"/>
-        <v>-2.6903800000000002</v>
+        <f>H15/1000000</f>
+        <v>-4.0206400000000002</v>
       </c>
       <c r="T15" s="5">
         <f t="shared" si="4"/>
-        <v>-4.2001499999999998</v>
+        <v>-4.2079000000000004</v>
       </c>
       <c r="U15" s="2">
         <f t="shared" si="5"/>
-        <v>-17.595600000000001</v>
+        <v>-14.594799999999999</v>
       </c>
       <c r="W15" s="3">
-        <f t="shared" ref="W15:X23" si="7">W14+M15</f>
+        <f t="shared" ref="W15:X23" si="9">W14+M15</f>
         <v>-3.3242600300000005</v>
       </c>
       <c r="X15" s="3">
-        <f t="shared" si="7"/>
-        <v>-3.3242600300000005</v>
+        <f t="shared" si="9"/>
+        <v>-6.8700630300000007</v>
       </c>
       <c r="Y15" s="3">
-        <f t="shared" ref="Y15:Y23" si="8">Y14+O15</f>
-        <v>-7.3196830300000002</v>
+        <f t="shared" ref="Y15:Y23" si="10">Y14+O15</f>
+        <v>-7.3403230300000004</v>
       </c>
       <c r="Z15" s="4">
         <f>Z14+P15</f>
-        <v>-43.054133030000003</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+        <v>-35.055633029999996</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>13</v>
       </c>
@@ -4244,10 +4253,10 @@
         <v>-2358840</v>
       </c>
       <c r="H16" s="1">
-        <v>-2086150</v>
+        <v>-3416410</v>
       </c>
       <c r="J16" s="1">
-        <v>-16707400</v>
+        <v>-13706600</v>
       </c>
       <c r="L16">
         <v>13</v>
@@ -4274,8 +4283,8 @@
         <v>-2.3588399999999998</v>
       </c>
       <c r="S16" s="2">
-        <f t="shared" si="3"/>
-        <v>-2.0861499999999999</v>
+        <f>H16/1000000</f>
+        <v>-3.4164099999999999</v>
       </c>
       <c r="T16" s="2">
         <f t="shared" si="4"/>
@@ -4283,26 +4292,26 @@
       </c>
       <c r="U16" s="2">
         <f t="shared" si="5"/>
-        <v>-16.7074</v>
+        <v>-13.7066</v>
       </c>
       <c r="W16" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-2.3005200300000004</v>
       </c>
       <c r="X16" s="3">
-        <f t="shared" si="7"/>
-        <v>-1.4585200300000005</v>
+        <f t="shared" si="9"/>
+        <v>-5.004323030000001</v>
       </c>
       <c r="Y16" s="3">
-        <f t="shared" si="8"/>
-        <v>-7.3196830300000002</v>
+        <f t="shared" si="10"/>
+        <v>-7.3403230300000004</v>
       </c>
       <c r="Z16" s="3">
-        <f t="shared" ref="Z16:Z23" si="9">Z15+P16</f>
-        <v>-40.31151303</v>
-      </c>
-    </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" ref="Z16:Z23" si="11">Z15+P16</f>
+        <v>-32.313013029999993</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>14</v>
       </c>
@@ -4310,7 +4319,7 @@
         <v>948880</v>
       </c>
       <c r="C17" s="1">
-        <v>1799270</v>
+        <v>1799260</v>
       </c>
       <c r="E17" s="1">
         <v>2734160</v>
@@ -4319,10 +4328,10 @@
         <v>-2077070</v>
       </c>
       <c r="H17" s="1">
-        <v>-1551860</v>
+        <v>-2882120</v>
       </c>
       <c r="J17" s="1">
-        <v>-15895500</v>
+        <v>-12894700</v>
       </c>
       <c r="L17">
         <v>14</v>
@@ -4333,7 +4342,7 @@
       </c>
       <c r="N17" s="2">
         <f t="shared" si="0"/>
-        <v>1.7992699999999999</v>
+        <v>1.7992600000000001</v>
       </c>
       <c r="O17" s="2">
         <f t="shared" si="1"/>
@@ -4349,8 +4358,8 @@
         <v>-2.07707</v>
       </c>
       <c r="S17" s="2">
-        <f t="shared" si="3"/>
-        <v>-1.55186</v>
+        <f>H17/1000000</f>
+        <v>-2.88212</v>
       </c>
       <c r="T17" s="2">
         <f t="shared" si="4"/>
@@ -4358,26 +4367,26 @@
       </c>
       <c r="U17" s="2">
         <f t="shared" si="5"/>
-        <v>-15.8955</v>
+        <v>-12.8947</v>
       </c>
       <c r="W17" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-1.3516400300000004</v>
       </c>
       <c r="X17" s="3">
-        <f t="shared" si="7"/>
-        <v>0.3407499699999994</v>
+        <f t="shared" si="9"/>
+        <v>-3.2050630300000007</v>
       </c>
       <c r="Y17" s="3">
-        <f t="shared" si="8"/>
-        <v>-7.3196830300000002</v>
+        <f t="shared" si="10"/>
+        <v>-7.3403230300000004</v>
       </c>
       <c r="Z17" s="3">
-        <f t="shared" si="9"/>
-        <v>-37.577353029999998</v>
-      </c>
-    </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" si="11"/>
+        <v>-29.578853029999994</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>15</v>
       </c>
@@ -4394,10 +4403,10 @@
         <v>-1839550</v>
       </c>
       <c r="H18" s="1">
-        <v>-1080490</v>
+        <v>-2410750</v>
       </c>
       <c r="J18" s="1">
-        <v>-15153500</v>
+        <v>-12152700</v>
       </c>
       <c r="L18">
         <v>15</v>
@@ -4424,8 +4433,8 @@
         <v>-1.83955</v>
       </c>
       <c r="S18" s="2">
-        <f t="shared" si="3"/>
-        <v>-1.08049</v>
+        <f>H18/1000000</f>
+        <v>-2.4107500000000002</v>
       </c>
       <c r="T18" s="2">
         <f t="shared" si="4"/>
@@ -4433,26 +4442,26 @@
       </c>
       <c r="U18" s="2">
         <f t="shared" si="5"/>
-        <v>-15.153499999999999</v>
+        <v>-12.152699999999999</v>
       </c>
       <c r="W18" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>-0.47931203000000044</v>
       </c>
       <c r="X18" s="3">
-        <f t="shared" si="7"/>
-        <v>2.0719299699999993</v>
+        <f t="shared" si="9"/>
+        <v>-1.4738830300000008</v>
       </c>
       <c r="Y18" s="3">
-        <f t="shared" si="8"/>
-        <v>-7.3196830300000002</v>
+        <f t="shared" si="10"/>
+        <v>-7.3403230300000004</v>
       </c>
       <c r="Z18" s="3">
-        <f t="shared" si="9"/>
-        <v>-34.852203029999998</v>
-      </c>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" si="11"/>
+        <v>-26.853703029999995</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>16</v>
       </c>
@@ -4469,10 +4478,10 @@
         <v>-1643940</v>
       </c>
       <c r="H19" s="1">
-        <v>-668333</v>
+        <v>-1998590</v>
       </c>
       <c r="J19" s="1">
-        <v>-14478100</v>
+        <v>-11477400</v>
       </c>
       <c r="L19">
         <v>16</v>
@@ -4499,8 +4508,8 @@
         <v>-1.64394</v>
       </c>
       <c r="S19" s="2">
-        <f t="shared" si="3"/>
-        <v>-0.66833299999999995</v>
+        <f>H19/1000000</f>
+        <v>-1.9985900000000001</v>
       </c>
       <c r="T19" s="2">
         <f t="shared" si="4"/>
@@ -4508,26 +4517,26 @@
       </c>
       <c r="U19" s="2">
         <f t="shared" si="5"/>
-        <v>-14.4781</v>
+        <v>-11.477399999999999</v>
       </c>
       <c r="W19" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.3041599699999995</v>
       </c>
       <c r="X19" s="3">
-        <f t="shared" si="7"/>
-        <v>3.7228099699999992</v>
+        <f t="shared" si="9"/>
+        <v>0.17699696999999914</v>
       </c>
       <c r="Y19" s="3">
-        <f t="shared" si="8"/>
-        <v>-7.3196830300000002</v>
+        <f t="shared" si="10"/>
+        <v>-7.3403230300000004</v>
       </c>
       <c r="Z19" s="3">
-        <f t="shared" si="9"/>
-        <v>-32.147223029999999</v>
-      </c>
-    </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" si="11"/>
+        <v>-24.148723029999996</v>
+      </c>
+    </row>
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>17</v>
       </c>
@@ -4544,10 +4553,10 @@
         <v>-1485340</v>
       </c>
       <c r="H20" s="1">
-        <v>-309185</v>
+        <v>-1639440</v>
       </c>
       <c r="J20" s="1">
-        <v>-13863700</v>
+        <v>-10862900</v>
       </c>
       <c r="L20">
         <v>17</v>
@@ -4574,8 +4583,8 @@
         <v>-1.4853400000000001</v>
       </c>
       <c r="S20" s="2">
-        <f t="shared" si="3"/>
-        <v>-0.30918499999999999</v>
+        <f>H20/1000000</f>
+        <v>-1.63944</v>
       </c>
       <c r="T20" s="2">
         <f t="shared" si="4"/>
@@ -4583,26 +4592,26 @@
       </c>
       <c r="U20" s="2">
         <f t="shared" si="5"/>
-        <v>-13.8637</v>
+        <v>-10.8629</v>
       </c>
       <c r="W20" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>0.9969879699999995</v>
       </c>
       <c r="X20" s="3">
-        <f t="shared" si="7"/>
-        <v>5.2916799699999988</v>
+        <f t="shared" si="9"/>
+        <v>1.7458669699999991</v>
       </c>
       <c r="Y20" s="3">
-        <f t="shared" si="8"/>
-        <v>-7.3196830300000002</v>
+        <f t="shared" si="10"/>
+        <v>-7.3403230300000004</v>
       </c>
       <c r="Z20" s="3">
-        <f t="shared" si="9"/>
-        <v>-29.463003029999999</v>
-      </c>
-    </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" si="11"/>
+        <v>-21.464503029999996</v>
+      </c>
+    </row>
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>18</v>
       </c>
@@ -4619,10 +4628,10 @@
         <v>-1357140</v>
       </c>
       <c r="H21" s="1">
-        <v>4734.1499999999996</v>
+        <v>-1325520</v>
       </c>
       <c r="J21" s="1">
-        <v>-13302500</v>
+        <v>-10301800</v>
       </c>
       <c r="L21">
         <v>18</v>
@@ -4649,8 +4658,8 @@
         <v>-1.35714</v>
       </c>
       <c r="S21" s="2">
-        <f t="shared" si="3"/>
-        <v>4.7341499999999995E-3</v>
+        <f>H21/1000000</f>
+        <v>-1.32552</v>
       </c>
       <c r="T21" s="2">
         <f t="shared" si="4"/>
@@ -4658,26 +4667,26 @@
       </c>
       <c r="U21" s="2">
         <f t="shared" si="5"/>
-        <v>-13.3025</v>
+        <v>-10.3018</v>
       </c>
       <c r="W21" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>1.6077639699999995</v>
       </c>
       <c r="X21" s="3">
-        <f t="shared" si="7"/>
-        <v>6.7872199699999989</v>
+        <f t="shared" si="9"/>
+        <v>3.241406969999999</v>
       </c>
       <c r="Y21" s="3">
-        <f t="shared" si="8"/>
-        <v>-7.3196830300000002</v>
+        <f t="shared" si="10"/>
+        <v>-7.3403230300000004</v>
       </c>
       <c r="Z21" s="3">
-        <f t="shared" si="9"/>
-        <v>-26.78975303</v>
-      </c>
-    </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" si="11"/>
+        <v>-18.791253029999996</v>
+      </c>
+    </row>
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>19</v>
       </c>
@@ -4694,10 +4703,10 @@
         <v>-1255740</v>
       </c>
       <c r="H22" s="1">
-        <v>278115</v>
+        <v>-1052140</v>
       </c>
       <c r="J22" s="1">
-        <v>-12790300</v>
+        <v>-9789500</v>
       </c>
       <c r="L22">
         <v>19</v>
@@ -4724,8 +4733,8 @@
         <v>-1.2557400000000001</v>
       </c>
       <c r="S22" s="2">
-        <f t="shared" si="3"/>
-        <v>0.278115</v>
+        <f>H22/1000000</f>
+        <v>-1.0521400000000001</v>
       </c>
       <c r="T22" s="2">
         <f t="shared" si="4"/>
@@ -4733,26 +4742,26 @@
       </c>
       <c r="U22" s="2">
         <f t="shared" si="5"/>
-        <v>-12.7903</v>
+        <v>-9.7895000000000003</v>
       </c>
       <c r="W22" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>2.1346019699999994</v>
       </c>
       <c r="X22" s="3">
-        <f t="shared" si="7"/>
-        <v>8.2076199699999997</v>
+        <f t="shared" si="9"/>
+        <v>4.6618069699999989</v>
       </c>
       <c r="Y22" s="3">
-        <f t="shared" si="8"/>
-        <v>-7.3196830300000002</v>
+        <f t="shared" si="10"/>
+        <v>-7.3403230300000004</v>
       </c>
       <c r="Z22" s="3">
-        <f t="shared" si="9"/>
-        <v>-24.12815303</v>
-      </c>
-    </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" si="11"/>
+        <v>-16.129653029999997</v>
+      </c>
+    </row>
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>20</v>
       </c>
@@ -4768,11 +4777,11 @@
       <c r="G23" s="1">
         <v>-1177910</v>
       </c>
-      <c r="H23" s="1">
-        <v>515202</v>
+      <c r="H23">
+        <v>-815057</v>
       </c>
       <c r="J23" s="1">
-        <v>-12322700</v>
+        <v>-9321960</v>
       </c>
       <c r="L23">
         <v>20</v>
@@ -4799,8 +4808,8 @@
         <v>-1.17791</v>
       </c>
       <c r="S23" s="2">
-        <f t="shared" si="3"/>
-        <v>0.51520200000000005</v>
+        <f>H23/1000000</f>
+        <v>-0.81505700000000003</v>
       </c>
       <c r="T23" s="2">
         <f t="shared" si="4"/>
@@ -4808,26 +4817,26 @@
       </c>
       <c r="U23" s="2">
         <f t="shared" si="5"/>
-        <v>-12.322699999999999</v>
+        <v>-9.3219600000000007</v>
       </c>
       <c r="W23" s="3">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>2.5755829699999992</v>
       </c>
       <c r="X23" s="3">
-        <f t="shared" si="7"/>
-        <v>9.551059969999999</v>
+        <f t="shared" si="9"/>
+        <v>6.0052469699999991</v>
       </c>
       <c r="Y23" s="3">
-        <f t="shared" si="8"/>
-        <v>-7.3196830300000002</v>
+        <f t="shared" si="10"/>
+        <v>-7.3403230300000004</v>
       </c>
       <c r="Z23" s="3">
-        <f t="shared" si="9"/>
-        <v>-21.478893030000002</v>
-      </c>
-    </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.3">
+        <f t="shared" si="11"/>
+        <v>-13.480393029999997</v>
+      </c>
+    </row>
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>21</v>
       </c>
@@ -4843,11 +4852,11 @@
       <c r="G24" s="1">
         <v>-1121760</v>
       </c>
-      <c r="H24" s="1">
-        <v>718843</v>
+      <c r="H24">
+        <v>-611416</v>
       </c>
       <c r="J24" s="1">
-        <v>-11897100</v>
+        <v>-8896370</v>
       </c>
       <c r="L24">
         <v>21</v>
@@ -4874,8 +4883,8 @@
         <v>-1.1217600000000001</v>
       </c>
       <c r="S24" s="2">
-        <f t="shared" si="3"/>
-        <v>0.71884300000000001</v>
+        <f>H24/1000000</f>
+        <v>-0.61141599999999996</v>
       </c>
       <c r="T24" s="2">
         <f t="shared" si="4"/>
@@ -4883,10 +4892,10 @@
       </c>
       <c r="U24" s="2">
         <f t="shared" si="5"/>
-        <v>-11.8971</v>
-      </c>
-    </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.3">
+        <v>-8.8963699999999992</v>
+      </c>
+    </row>
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>22</v>
       </c>
@@ -4902,11 +4911,11 @@
       <c r="G25" s="1">
         <v>-1084510</v>
       </c>
-      <c r="H25" s="1">
-        <v>892676</v>
+      <c r="H25">
+        <v>-437583</v>
       </c>
       <c r="J25" s="1">
-        <v>-11509900</v>
+        <v>-8509080</v>
       </c>
       <c r="L25">
         <v>22</v>
@@ -4933,8 +4942,8 @@
         <v>-1.0845100000000001</v>
       </c>
       <c r="S25" s="2">
-        <f t="shared" si="3"/>
-        <v>0.89267600000000003</v>
+        <f>H25/1000000</f>
+        <v>-0.437583</v>
       </c>
       <c r="T25" s="2">
         <f t="shared" si="4"/>
@@ -4942,10 +4951,10 @@
       </c>
       <c r="U25" s="2">
         <f t="shared" si="5"/>
-        <v>-11.5099</v>
-      </c>
-    </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.3">
+        <v>-8.5090800000000009</v>
+      </c>
+    </row>
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>23</v>
       </c>
@@ -4961,11 +4970,11 @@
       <c r="G26" s="1">
         <v>-1062840</v>
       </c>
-      <c r="H26" s="1">
-        <v>1040820</v>
+      <c r="H26">
+        <v>-289439</v>
       </c>
       <c r="J26" s="1">
-        <v>-11156700</v>
+        <v>-8155950</v>
       </c>
       <c r="L26">
         <v>23</v>
@@ -4992,8 +5001,8 @@
         <v>-1.06284</v>
       </c>
       <c r="S26" s="5">
-        <f t="shared" si="3"/>
-        <v>1.0408200000000001</v>
+        <f>H26/1000000</f>
+        <v>-0.289439</v>
       </c>
       <c r="T26" s="2">
         <f t="shared" si="4"/>
@@ -5001,10 +5010,10 @@
       </c>
       <c r="U26" s="5">
         <f t="shared" si="5"/>
-        <v>-11.156700000000001</v>
-      </c>
-    </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.3">
+        <v>-8.1559500000000007</v>
+      </c>
+    </row>
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>24</v>
       </c>
@@ -5020,11 +5029,11 @@
       <c r="G27" s="1">
         <v>-1054680</v>
       </c>
-      <c r="H27" s="1">
-        <v>1166100</v>
+      <c r="H27">
+        <v>-164159</v>
       </c>
       <c r="J27" s="1">
-        <v>-10834800</v>
+        <v>-7834050</v>
       </c>
       <c r="L27">
         <v>24</v>
@@ -5051,8 +5060,8 @@
         <v>-1.0546800000000001</v>
       </c>
       <c r="S27" s="2">
-        <f t="shared" si="3"/>
-        <v>1.1660999999999999</v>
+        <f>H27/1000000</f>
+        <v>-0.164159</v>
       </c>
       <c r="T27" s="2">
         <f t="shared" si="4"/>
@@ -5060,10 +5069,10 @@
       </c>
       <c r="U27" s="2">
         <f t="shared" si="5"/>
-        <v>-10.8348</v>
-      </c>
-    </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.3">
+        <v>-7.8340500000000004</v>
+      </c>
+    </row>
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>25</v>
       </c>
@@ -5079,11 +5088,11 @@
       <c r="G28" s="1">
         <v>-980417</v>
       </c>
-      <c r="H28" s="1">
-        <v>1348820</v>
+      <c r="H28">
+        <v>18563.7</v>
       </c>
       <c r="J28" s="1">
-        <v>-10463700</v>
+        <v>-7462960</v>
       </c>
       <c r="L28">
         <v>25</v>
@@ -5110,8 +5119,8 @@
         <v>-0.98041699999999998</v>
       </c>
       <c r="S28" s="2">
-        <f t="shared" si="3"/>
-        <v>1.3488199999999999</v>
+        <f>H28/1000000</f>
+        <v>1.8563700000000002E-2</v>
       </c>
       <c r="T28" s="2">
         <f t="shared" si="4"/>
@@ -5119,8 +5128,341 @@
       </c>
       <c r="U28" s="2">
         <f t="shared" si="5"/>
-        <v>-10.463699999999999</v>
-      </c>
+        <v>-7.4629599999999998</v>
+      </c>
+    </row>
+    <row r="33" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J33" t="s">
+        <v>11</v>
+      </c>
+      <c r="K33" t="s">
+        <v>13</v>
+      </c>
+      <c r="L33" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J34">
+        <v>1</v>
+      </c>
+      <c r="K34" s="1">
+        <v>-13557300</v>
+      </c>
+      <c r="L34" s="1">
+        <v>-13557300</v>
+      </c>
+    </row>
+    <row r="35" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J35">
+        <v>2</v>
+      </c>
+      <c r="K35" s="1">
+        <v>-4423200</v>
+      </c>
+      <c r="L35" s="1">
+        <v>9961670</v>
+      </c>
+    </row>
+    <row r="36" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J36">
+        <v>3</v>
+      </c>
+      <c r="K36" s="1">
+        <v>-2528160</v>
+      </c>
+      <c r="L36" s="1">
+        <v>2253980</v>
+      </c>
+    </row>
+    <row r="37" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J37">
+        <v>4</v>
+      </c>
+      <c r="K37" s="1">
+        <v>-1520630</v>
+      </c>
+      <c r="L37" s="1">
+        <v>1306930</v>
+      </c>
+    </row>
+    <row r="38" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J38">
+        <v>5</v>
+      </c>
+      <c r="K38" s="1">
+        <v>-1042570</v>
+      </c>
+      <c r="L38" s="1">
+        <v>676313</v>
+      </c>
+    </row>
+    <row r="39" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J39">
+        <v>6</v>
+      </c>
+      <c r="K39" s="1">
+        <v>-703987</v>
+      </c>
+      <c r="L39" s="1">
+        <v>522382</v>
+      </c>
+    </row>
+    <row r="40" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J40">
+        <v>7</v>
+      </c>
+      <c r="K40" s="1">
+        <v>-702556</v>
+      </c>
+      <c r="L40" s="1">
+        <v>2407.9699999999998</v>
+      </c>
+    </row>
+    <row r="41" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J41">
+        <v>8</v>
+      </c>
+      <c r="K41">
+        <v>-987222</v>
+      </c>
+      <c r="L41" s="1">
+        <v>-522389</v>
+      </c>
+    </row>
+    <row r="42" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J42">
+        <v>9</v>
+      </c>
+      <c r="K42" s="1">
+        <v>-1332610</v>
+      </c>
+      <c r="L42" s="1">
+        <v>-691240</v>
+      </c>
+    </row>
+    <row r="43" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J43">
+        <v>10</v>
+      </c>
+      <c r="K43" s="1">
+        <v>-1729280</v>
+      </c>
+      <c r="L43" s="1">
+        <v>-865807</v>
+      </c>
+    </row>
+    <row r="44" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J44" s="1">
+        <v>11</v>
+      </c>
+      <c r="K44" s="1">
+        <v>-2168900</v>
+      </c>
+      <c r="L44" s="1">
+        <v>-1046480</v>
+      </c>
+    </row>
+    <row r="45" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J45" s="1">
+        <v>12</v>
+      </c>
+      <c r="K45" s="1">
+        <v>-11035600</v>
+      </c>
+      <c r="L45" s="1">
+        <v>-23018800</v>
+      </c>
+    </row>
+    <row r="46" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J46" s="1">
+        <v>13</v>
+      </c>
+      <c r="K46" s="1">
+        <v>-14594800</v>
+      </c>
+      <c r="L46" s="1">
+        <v>-10077300</v>
+      </c>
+    </row>
+    <row r="47" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J47" s="1">
+        <v>14</v>
+      </c>
+      <c r="K47" s="1">
+        <v>-13706600</v>
+      </c>
+      <c r="L47" s="1">
+        <v>2742620</v>
+      </c>
+    </row>
+    <row r="48" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J48">
+        <v>15</v>
+      </c>
+      <c r="K48" s="1">
+        <v>-12894700</v>
+      </c>
+      <c r="L48" s="1">
+        <v>2734160</v>
+      </c>
+    </row>
+    <row r="49" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J49">
+        <v>16</v>
+      </c>
+      <c r="K49" s="1">
+        <v>-12152700</v>
+      </c>
+      <c r="L49" s="1">
+        <v>2725150</v>
+      </c>
+    </row>
+    <row r="50" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J50">
+        <v>17</v>
+      </c>
+      <c r="K50" s="1">
+        <v>-11477400</v>
+      </c>
+      <c r="L50" s="1">
+        <v>2704980</v>
+      </c>
+    </row>
+    <row r="51" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J51">
+        <v>18</v>
+      </c>
+      <c r="K51" s="1">
+        <v>-10862900</v>
+      </c>
+      <c r="L51" s="1">
+        <v>2684220</v>
+      </c>
+    </row>
+    <row r="52" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J52">
+        <v>19</v>
+      </c>
+      <c r="K52" s="1">
+        <v>-10301800</v>
+      </c>
+      <c r="L52" s="1">
+        <v>2673250</v>
+      </c>
+    </row>
+    <row r="53" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J53">
+        <v>20</v>
+      </c>
+      <c r="K53" s="1">
+        <v>-9789500</v>
+      </c>
+      <c r="L53" s="1">
+        <v>2661600</v>
+      </c>
+    </row>
+    <row r="54" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J54" s="1">
+        <v>21</v>
+      </c>
+      <c r="K54" s="1">
+        <v>-9321960</v>
+      </c>
+      <c r="L54" s="1">
+        <v>2649260</v>
+      </c>
+    </row>
+    <row r="55" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J55" s="1">
+        <v>22</v>
+      </c>
+      <c r="K55" s="1">
+        <v>-8896370</v>
+      </c>
+      <c r="L55" s="1">
+        <v>2630080</v>
+      </c>
+    </row>
+    <row r="56" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J56">
+        <v>23</v>
+      </c>
+      <c r="K56" s="1">
+        <v>-8509080</v>
+      </c>
+      <c r="L56" s="1">
+        <v>2610170</v>
+      </c>
+    </row>
+    <row r="57" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J57" s="1">
+        <v>24</v>
+      </c>
+      <c r="K57" s="1">
+        <v>-8155950</v>
+      </c>
+      <c r="L57" s="1">
+        <v>2595680</v>
+      </c>
+    </row>
+    <row r="58" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J58" s="1">
+        <v>25</v>
+      </c>
+      <c r="K58" s="1">
+        <v>-7834050</v>
+      </c>
+      <c r="L58" s="1">
+        <v>2580430</v>
+      </c>
+    </row>
+    <row r="59" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J59" s="1">
+        <v>26</v>
+      </c>
+      <c r="K59" s="1">
+        <v>-7462960</v>
+      </c>
+      <c r="L59" s="1">
+        <v>3244240</v>
+      </c>
+    </row>
+    <row r="60" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J60" s="1"/>
+      <c r="K60" s="1"/>
+    </row>
+    <row r="61" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J61" s="1"/>
+      <c r="K61" s="1"/>
+    </row>
+    <row r="62" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J62" s="1"/>
+      <c r="K62" s="1"/>
+    </row>
+    <row r="63" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J63" s="1"/>
+    </row>
+    <row r="64" spans="10:12" x14ac:dyDescent="0.25">
+      <c r="J64" s="1"/>
+    </row>
+    <row r="65" spans="10:11" x14ac:dyDescent="0.25">
+      <c r="J65" s="1"/>
+    </row>
+    <row r="66" spans="10:11" x14ac:dyDescent="0.25">
+      <c r="J66" s="1"/>
+    </row>
+    <row r="67" spans="10:11" x14ac:dyDescent="0.25">
+      <c r="J67" s="1"/>
+      <c r="K67" s="1"/>
+    </row>
+    <row r="68" spans="10:11" x14ac:dyDescent="0.25">
+      <c r="J68" s="1"/>
+      <c r="K68" s="1"/>
+    </row>
+    <row r="69" spans="10:11" x14ac:dyDescent="0.25">
+      <c r="J69" s="1"/>
+      <c r="K69" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5140,6 +5482,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A788E4FEB44D0B4CB1AD2E9A3A83F076" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c1d34d9b8e131c103df8a093e310b027">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8baa01ab-7cf8-4360-9f3f-f87b1ec95c26" xmlns:ns3="d481fc2a-e230-47f7-a716-4f7f4b27a8e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c44e149c0724d485dcb6f09127e30ffd" ns2:_="" ns3:_="">
     <xsd:import namespace="8baa01ab-7cf8-4360-9f3f-f87b1ec95c26"/>
@@ -5368,15 +5719,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A82D478-F143-4E1A-BE03-DF93E0476218}">
   <ds:schemaRefs>
@@ -5389,6 +5731,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CB2C9E99-917F-4BDF-B9E4-ADA5D0AFF133}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F33A64FD-BD8E-4A10-881A-543F22FB0B66}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5407,14 +5757,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CB2C9E99-917F-4BDF-B9E4-ADA5D0AFF133}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{95965d95-ecc0-4720-b759-1f33c42ed7da}" enabled="1" method="Standard" siteId="{a0f29d7e-28cd-4f54-8442-7885aee7c080}" removed="0"/>

</xml_diff>